<commit_message>
Regenera artefactos BAU como prueba del flujo run.py con snapshot post-A2
Corrida de run.py end-to-end con los cambios del commit anterior:
- A2 crea por primera vez A1_Outputs/_post_a2_snapshot_BAU/ (8 xlsx).
- A3 restaura desde el snapshot y regenera A1_Outputs/A1_Outputs_BAU/.
- B1/B2 producen los CSVs de A2_Output_Params/BAU/ y el cplex.log.

Sirve como punto de partida reproducible: futuras corridas de run.py en clones
frescos detectarán el snapshot y omitirán A1+A2.
</commit_message>
<xml_diff>
--- a/t1_confection/A1_Outputs/A1_Outputs_BAU/A-O_AR_Model_Base_Year.xlsx
+++ b/t1_confection/A1_Outputs/A1_Outputs_BAU/A-O_AR_Model_Base_Year.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="5" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Primary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Secondary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Demand Techs" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Distribution Transport" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transport" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transport Groups" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Primary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Secondary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Demand Techs" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Distribution Transport" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Transport" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Transport Groups" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Fix stage 6 persist_restrictions y regenera artefactos BAU
- A3_process.py: stage_6_persist_restrictions buscaba *_CHANGES.json dentro
  de stage5/, pero el rules_script lo escribe como sibling en el workdir
  (s5.parent). Corrige la busqueda usando el patron <s5.name>_PRE_*_CHANGES.json
  con fallback al glob generico. Sin este fix las Restrictions nunca se
  persistian a SOASIA v18 tras cada run.
- SOASIA_OSeMOSYS_Template_v18.xlsx: hoja Restrictions ahora contiene las
  1960 filas escritas por el lid_rule en la corrida BAU.
- A1_Outputs_BAU/: regenerados con la version corregida del pipeline
  multi-escenario end-to-end (tests 1, 4, 5, 6, 7, 8 del plan validados).
</commit_message>
<xml_diff>
--- a/t1_confection/A1_Outputs/A1_Outputs_BAU/A-O_AR_Model_Base_Year.xlsx
+++ b/t1_confection/A1_Outputs/A1_Outputs_BAU/A-O_AR_Model_Base_Year.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="5" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Primary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Secondary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Demand Techs" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Distribution Transport" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Transport" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Transport Groups" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Primary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Secondary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Demand Techs" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Distribution Transport" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transport" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transport Groups" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Regenera artefactos A1_Outputs_BAU con cadena multi-script
</commit_message>
<xml_diff>
--- a/t1_confection/A1_Outputs/A1_Outputs_BAU/A-O_AR_Model_Base_Year.xlsx
+++ b/t1_confection/A1_Outputs/A1_Outputs_BAU/A-O_AR_Model_Base_Year.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="5" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Primary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Secondary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Demand Techs" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Distribution Transport" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transport" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transport Groups" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Primary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Secondary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Demand Techs" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Distribution Transport" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Transport" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Transport Groups" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
chore: checkpoint constrained runs with pending B_OptVRE backstop fix
Checkpoint updated constrained runs for the 3-scenario baseline.

Current status:
- BAU ran with the updated constraints.
- A_Calibrated_BAU ran with the updated constraints.
- B_Optimised_VRE ran with the updated constraints, but still has pending backstop activation to remove in 3 regions during the final 3 years.

This preserves the current hard-to-reproduce run state before applying the final B_Optimised_VRE backstop correction.
</commit_message>
<xml_diff>
--- a/t1_confection/A1_Outputs/A1_Outputs_BAU/A-O_AR_Model_Base_Year.xlsx
+++ b/t1_confection/A1_Outputs/A1_Outputs_BAU/A-O_AR_Model_Base_Year.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="5" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Primary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Secondary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Demand Techs" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Distribution Transport" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Transport" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Transport Groups" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Primary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Secondary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Demand Techs" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Distribution Transport" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transport" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transport Groups" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>

</xml_diff>